<commit_message>
passada melhorias e refatoracao
</commit_message>
<xml_diff>
--- a/utils/monday_sprint_2023-t1.xlsx
+++ b/utils/monday_sprint_2023-t1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
   <si>
     <t>Ticket</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Equipe TI</t>
   </si>
   <si>
-    <t>Abertura</t>
+    <t>Entrada Sprint</t>
   </si>
   <si>
     <t>Encerramento</t>
@@ -51,6 +51,9 @@
     <t>Status</t>
   </si>
   <si>
+    <t>SLA (15 dias)</t>
+  </si>
+  <si>
     <t>Semana</t>
   </si>
   <si>
@@ -60,51 +63,57 @@
     <t>19258</t>
   </si>
   <si>
+    <t>Usinagem</t>
+  </si>
+  <si>
+    <t>Melhoria</t>
+  </si>
+  <si>
+    <t>Solicitação de serviço</t>
+  </si>
+  <si>
+    <t>Integração CRP e ERP</t>
+  </si>
+  <si>
+    <t>Bom dia, Segue abaixo chamado referente a integração entre o CRP e o ERP Altona. * Enviar o registro para o CRP no momento da criação da etiqueta (azul). Att,</t>
+  </si>
+  <si>
+    <t>Média</t>
+  </si>
+  <si>
+    <t>Caio Henrique Vicente Bento</t>
+  </si>
+  <si>
+    <t>Sistemas</t>
+  </si>
+  <si>
+    <t>06/04/2023</t>
+  </si>
+  <si>
+    <t>04/05/2026</t>
+  </si>
+  <si>
+    <t>Fila</t>
+  </si>
+  <si>
+    <t>Aberto</t>
+  </si>
+  <si>
+    <t>Semana 1</t>
+  </si>
+  <si>
+    <t>Abril</t>
+  </si>
+  <si>
+    <t>Dashboard de Change Log - Governança de TI</t>
+  </si>
+  <si>
+    <t>Período</t>
+  </si>
+  <si>
     <t>2023-T1</t>
   </si>
   <si>
-    <t>Melhoria</t>
-  </si>
-  <si>
-    <t>Solicitação de serviço</t>
-  </si>
-  <si>
-    <t>Integração CRP e ERP</t>
-  </si>
-  <si>
-    <t>Bom dia, Segue abaixo chamado referente a integração entre o CRP e o ERP Altona. * Enviar o registro para o CRP no momento da criação da etiqueta (azul). Att,</t>
-  </si>
-  <si>
-    <t>Média</t>
-  </si>
-  <si>
-    <t>Caio Henrique Vicente Bento</t>
-  </si>
-  <si>
-    <t>Sistemas</t>
-  </si>
-  <si>
-    <t>17/03/2023</t>
-  </si>
-  <si>
-    <t>09/05/2026</t>
-  </si>
-  <si>
-    <t>Fila</t>
-  </si>
-  <si>
-    <t>Semana 3</t>
-  </si>
-  <si>
-    <t>Março</t>
-  </si>
-  <si>
-    <t>Dashboard de Change Log - Governança de TI</t>
-  </si>
-  <si>
-    <t>Período</t>
-  </si>
-  <si>
     <t>Base</t>
   </si>
   <si>
@@ -144,7 +153,7 @@
     <t>Distribuição por Tipo</t>
   </si>
   <si>
-    <t>Cumprimento SLA</t>
+    <t>Cumprimento SLA (15 dias)</t>
   </si>
   <si>
     <t>Status Final</t>
@@ -169,6 +178,9 @@
   </si>
   <si>
     <t>A fazer</t>
+  </si>
+  <si>
+    <t>Abertos</t>
   </si>
   <si>
     <t>Impedimento</t>
@@ -609,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -619,13 +631,15 @@
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="11" width="14" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -668,49 +682,55 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -726,23 +746,23 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>
@@ -750,16 +770,16 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -778,12 +798,12 @@
     </row>
     <row r="21" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J21" s="6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J22" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -791,7 +811,7 @@
     </row>
     <row r="23" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J23" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -799,7 +819,7 @@
     </row>
     <row r="24" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J24" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -817,7 +837,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -830,12 +850,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -859,54 +879,54 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="M10" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -914,19 +934,19 @@
     </row>
     <row r="11" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -934,13 +954,19 @@
     </row>
     <row r="12" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
+      <c r="J12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
       <c r="M12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -948,13 +974,13 @@
     </row>
     <row r="13" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="M13" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -962,13 +988,13 @@
     </row>
     <row r="14" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -976,7 +1002,7 @@
     </row>
     <row r="15" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M15" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -984,7 +1010,7 @@
     </row>
     <row r="16" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N16">
         <v>1</v>
@@ -992,7 +1018,7 @@
     </row>
     <row r="17" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M17" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1000,7 +1026,7 @@
     </row>
     <row r="19" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D19" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="4:7" x14ac:dyDescent="0.25">
@@ -1011,24 +1037,10 @@
         <v>1</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="4:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="2">
-        <v>1144</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Alterações na api de vinculação com o movidesk
</commit_message>
<xml_diff>
--- a/utils/monday_sprint_2023-t1.xlsx
+++ b/utils/monday_sprint_2023-t1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
   <si>
     <t>Ticket</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Equipe TI</t>
   </si>
   <si>
-    <t>Entrada Sprint</t>
+    <t>Abertura</t>
   </si>
   <si>
     <t>Encerramento</t>
@@ -51,7 +51,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>SLA (15 dias)</t>
+    <t>Dentro da SLA</t>
   </si>
   <si>
     <t>Semana</t>
@@ -96,7 +96,7 @@
     <t>Fila</t>
   </si>
   <si>
-    <t>Aberto</t>
+    <t>Não</t>
   </si>
   <si>
     <t>Semana 1</t>
@@ -111,7 +111,7 @@
     <t>Período</t>
   </si>
   <si>
-    <t>2023-T1</t>
+    <t>Abr/2023</t>
   </si>
   <si>
     <t>Base</t>
@@ -172,9 +172,6 @@
   </si>
   <si>
     <t>Alta</t>
-  </si>
-  <si>
-    <t>Não</t>
   </si>
   <si>
     <t>A fazer</t>
@@ -837,7 +834,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -940,13 +937,13 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
         <v>53</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="M11" t="s">
-        <v>54</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -960,13 +957,13 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
+        <v>54</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="M12" t="s">
         <v>55</v>
-      </c>
-      <c r="K12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>56</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -974,13 +971,13 @@
     </row>
     <row r="13" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G13" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="M13" t="s">
         <v>57</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="M13" t="s">
-        <v>58</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -988,7 +985,7 @@
     </row>
     <row r="14" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -1002,7 +999,7 @@
     </row>
     <row r="15" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -1018,7 +1015,7 @@
     </row>
     <row r="17" spans="13:14" x14ac:dyDescent="0.25">
       <c r="M17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1026,10 +1023,10 @@
     </row>
     <row r="19" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D19" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" spans="4:7" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D20" s="1" t="s">
         <v>0</v>
       </c>
@@ -1037,10 +1034,24 @@
         <v>1</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="4:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="2">
+        <v>1154</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>